<commit_message>
chore(catmat): update data sources
</commit_message>
<xml_diff>
--- a/scripts/catmat/_fontes/Margens.xlsx
+++ b/scripts/catmat/_fontes/Margens.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\DCOM - Geral\DCOM\R Scripts\CATMAT\_fontes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\DCOM - Geral\DCOM\compras-web\scripts\catmat\_fontes\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02B385F-3D15-4D74-8633-C9D33693BF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -3619,7 +3620,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -3817,7 +3818,7 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3919,9 +3920,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3959,9 +3960,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -3996,7 +3997,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4031,7 +4032,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4204,7 +4205,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F292"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -4723,7 +4724,7 @@
       <c r="E34" s="30"/>
       <c r="F34" s="30"/>
     </row>
-    <row r="35" spans="1:6" ht="75">
+    <row r="35" spans="1:6" ht="60">
       <c r="A35" s="3"/>
       <c r="B35" s="3" t="s">
         <v>51</v>
@@ -5349,7 +5350,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="105">
+    <row r="79" spans="1:6" ht="90">
       <c r="A79" s="3"/>
       <c r="B79" s="3" t="s">
         <v>96</v>
@@ -5829,7 +5830,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="120">
+    <row r="111" spans="1:6" ht="105">
       <c r="A111" s="3"/>
       <c r="B111" s="3" t="s">
         <v>126</v>
@@ -7409,7 +7410,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="210" spans="1:6" ht="135">
+    <row r="210" spans="1:6" ht="120">
       <c r="A210" s="10">
         <v>8531</v>
       </c>
@@ -8289,7 +8290,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="269" spans="1:6" ht="135">
+    <row r="269" spans="1:6" ht="120">
       <c r="A269" s="1" t="s">
         <v>272</v>
       </c>

</xml_diff>